<commit_message>
Output selection joint model
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
@@ -480,382 +480,382 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9.940793884389218e-15</v>
+        <v>4.333519793092376e-16</v>
       </c>
       <c r="B2" t="n">
-        <v>65.34293325112765</v>
+        <v>14.32970207851291</v>
       </c>
       <c r="C2" t="n">
-        <v>31.09242904364742</v>
+        <v>3.866825595790485</v>
       </c>
       <c r="D2" t="n">
-        <v>4.552802535897987</v>
+        <v>0.1867912526209001</v>
       </c>
       <c r="E2" t="n">
-        <v>0.2932054216663521</v>
+        <v>0.0008579083623691486</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>198.4616961007698</v>
+        <v>155.239055293018</v>
       </c>
       <c r="H2" t="n">
-        <v>442.9789105217176</v>
+        <v>268.7996574166283</v>
       </c>
       <c r="I2" t="n">
-        <v>475.7156190264243</v>
+        <v>120.7042447589839</v>
       </c>
       <c r="J2" t="n">
-        <v>416.0547430373032</v>
+        <v>232.2635270345889</v>
       </c>
       <c r="K2" t="n">
-        <v>259.5881299704866</v>
+        <v>324.7167866562738</v>
       </c>
       <c r="L2" t="n">
-        <v>207.5549464928588</v>
+        <v>172.3554033854167</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-1.211857004082994e-14</v>
+        <v>-4.626097186756907e-16</v>
       </c>
       <c r="B3" t="n">
-        <v>63.17971053312377</v>
+        <v>3.32380072754209</v>
       </c>
       <c r="C3" t="n">
-        <v>29.96411308237163</v>
+        <v>-3.612831347902668</v>
       </c>
       <c r="D3" t="n">
-        <v>4.011725325234443</v>
+        <v>0.01203443264648458</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2072849715388669</v>
+        <v>-0.0005248379813055048</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>292.6916163800972</v>
+        <v>126.298814844755</v>
       </c>
       <c r="H3" t="n">
-        <v>253.4092586536476</v>
+        <v>216.0676442175127</v>
       </c>
       <c r="I3" t="n">
-        <v>171.2688600913488</v>
+        <v>289.4538859265093</v>
       </c>
       <c r="J3" t="n">
-        <v>360.1673697718163</v>
+        <v>252.8933605583935</v>
       </c>
       <c r="K3" t="n">
-        <v>261.1959069984936</v>
+        <v>224.8385547745061</v>
       </c>
       <c r="L3" t="n">
-        <v>254.6744929531627</v>
+        <v>338.8836419862683</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>-1.202050186406843e-16</v>
+        <v>5.831630857015175e-18</v>
       </c>
       <c r="B4" t="n">
-        <v>66.02934538380599</v>
+        <v>18.22655570992734</v>
       </c>
       <c r="C4" t="n">
-        <v>31.20626981426283</v>
+        <v>5.055743683585101</v>
       </c>
       <c r="D4" t="n">
-        <v>4.627985916719141</v>
+        <v>0.1955330917041322</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01038044178291492</v>
+        <v>-0.007530158502224977</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>392.4576527544643</v>
+        <v>219.2313331751081</v>
       </c>
       <c r="H4" t="n">
-        <v>315.3133828712684</v>
+        <v>128.9995092647846</v>
       </c>
       <c r="I4" t="n">
-        <v>422.8719070916732</v>
+        <v>354.1295950808803</v>
       </c>
       <c r="J4" t="n">
-        <v>229.5465237936813</v>
+        <v>328.1288015049099</v>
       </c>
       <c r="K4" t="n">
-        <v>163.3831916726887</v>
+        <v>299.5968285520432</v>
       </c>
       <c r="L4" t="n">
-        <v>310.0181460888315</v>
+        <v>398.84889378004</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5.163206326778676e-16</v>
+        <v>1.660676677639394e-17</v>
       </c>
       <c r="B5" t="n">
-        <v>-65.90624776213046</v>
+        <v>-9.122017648126123</v>
       </c>
       <c r="C5" t="n">
-        <v>-31.08091462613098</v>
+        <v>-5.057369306583921</v>
       </c>
       <c r="D5" t="n">
-        <v>-4.628003896141625</v>
+        <v>-0.1961165214039462</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1471823220750438</v>
+        <v>0.00712352314118656</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>464.7851105829653</v>
+        <v>94.73192944856265</v>
       </c>
       <c r="H5" t="n">
-        <v>462.9870802959828</v>
+        <v>164.9460680543654</v>
       </c>
       <c r="I5" t="n">
-        <v>209.6939095995413</v>
+        <v>276.7068012752046</v>
       </c>
       <c r="J5" t="n">
-        <v>261.0271580505594</v>
+        <v>209.4676251409578</v>
       </c>
       <c r="K5" t="n">
-        <v>371.8833917410598</v>
+        <v>251.6464575009193</v>
       </c>
       <c r="L5" t="n">
-        <v>334.1153275320588</v>
+        <v>187.6528711351712</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-8.343678331145212e-18</v>
+        <v>-6.465077602175565e-17</v>
       </c>
       <c r="B6" t="n">
-        <v>24.34101662537363</v>
+        <v>12.54266116535535</v>
       </c>
       <c r="C6" t="n">
-        <v>31.23460795245</v>
+        <v>5.073828348551419</v>
       </c>
       <c r="D6" t="n">
-        <v>4.631316851653938</v>
+        <v>0.2028242187617373</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.1362989576572911</v>
+        <v>0.003783973571307417</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>160.1374851976115</v>
+        <v>203.0457747057284</v>
       </c>
       <c r="H6" t="n">
-        <v>199.4972526483417</v>
+        <v>102.6348062425755</v>
       </c>
       <c r="I6" t="n">
-        <v>183.430394755112</v>
+        <v>134.1890534089342</v>
       </c>
       <c r="J6" t="n">
-        <v>241.711525274946</v>
+        <v>323.3941416316508</v>
       </c>
       <c r="K6" t="n">
-        <v>379.3637988858356</v>
+        <v>194.0390985245222</v>
       </c>
       <c r="L6" t="n">
-        <v>345.8556050598332</v>
+        <v>459.24388744721</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1.014688373348133e-15</v>
+        <v>9.780957829962677e-17</v>
       </c>
       <c r="B7" t="n">
-        <v>-30.57030797746024</v>
+        <v>-8.714835450147174</v>
       </c>
       <c r="C7" t="n">
-        <v>-31.23457131638467</v>
+        <v>-5.073926494032001</v>
       </c>
       <c r="D7" t="n">
-        <v>-4.623845117484152</v>
+        <v>-0.202932551570449</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.2973545598157386</v>
+        <v>0.005647533378655745</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>342.7813656293661</v>
+        <v>209.1811638258204</v>
       </c>
       <c r="H7" t="n">
-        <v>183.1703678437171</v>
+        <v>264.6011480012432</v>
       </c>
       <c r="I7" t="n">
-        <v>292.7876326550343</v>
+        <v>143.6996660999505</v>
       </c>
       <c r="J7" t="n">
-        <v>427.4767156303036</v>
+        <v>269.6116397426714</v>
       </c>
       <c r="K7" t="n">
-        <v>307.5621396938427</v>
+        <v>336.58436347155</v>
       </c>
       <c r="L7" t="n">
-        <v>342.8459931841588</v>
+        <v>206.0342853507156</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8.229926309129317e-17</v>
+        <v>-1.092429492735409e-16</v>
       </c>
       <c r="B8" t="n">
-        <v>-27.66605975679562</v>
+        <v>13.85418898014175</v>
       </c>
       <c r="C8" t="n">
-        <v>1.067647483400888</v>
+        <v>1.16787605292904</v>
       </c>
       <c r="D8" t="n">
-        <v>4.633267345186171</v>
+        <v>0.2031241998160949</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.01674395573535175</v>
+        <v>0.0006447783890831559</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>244.8777788044186</v>
+        <v>114.651205812829</v>
       </c>
       <c r="H8" t="n">
-        <v>414.586869905781</v>
+        <v>252.8297301668283</v>
       </c>
       <c r="I8" t="n">
-        <v>198.9677921464707</v>
+        <v>323.0668816220197</v>
       </c>
       <c r="J8" t="n">
-        <v>193.4914271019785</v>
+        <v>357.506875532349</v>
       </c>
       <c r="K8" t="n">
-        <v>175.1605859195013</v>
+        <v>327.965826704513</v>
       </c>
       <c r="L8" t="n">
-        <v>271.7000874512382</v>
+        <v>194.9570618870869</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6.66682269851009e-17</v>
+        <v>3.633665321794214e-17</v>
       </c>
       <c r="B9" t="n">
-        <v>-42.42638830924984</v>
+        <v>11.01893040258089</v>
       </c>
       <c r="C9" t="n">
-        <v>-12.03506969916373</v>
+        <v>-1.671335538621919</v>
       </c>
       <c r="D9" t="n">
-        <v>-4.633474617794199</v>
+        <v>-0.2031258266151972</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.004670479181094366</v>
+        <v>1.785955698459928e-05</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>252.3577601870796</v>
+        <v>110.8629981366128</v>
       </c>
       <c r="H9" t="n">
-        <v>386.1080042037839</v>
+        <v>245.1752277991199</v>
       </c>
       <c r="I9" t="n">
-        <v>377.0751564747108</v>
+        <v>328.1722045891901</v>
       </c>
       <c r="J9" t="n">
-        <v>464.6846390562647</v>
+        <v>284.4744390318555</v>
       </c>
       <c r="K9" t="n">
-        <v>232.7650087767408</v>
+        <v>193.9427140627287</v>
       </c>
       <c r="L9" t="n">
-        <v>220.7429079866505</v>
+        <v>200.6697782694127</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.289258457479122e-16</v>
+        <v>-5.533198564341929e-17</v>
       </c>
       <c r="B10" t="n">
-        <v>11.17117782101327</v>
+        <v>-0.9036399014302505</v>
       </c>
       <c r="C10" t="n">
-        <v>-21.98828482354696</v>
+        <v>-2.837660219235009</v>
       </c>
       <c r="D10" t="n">
-        <v>4.617457403845774</v>
+        <v>-0.202955857918495</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3845803842123143</v>
+        <v>0.007829107217133075</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>327.4294104484989</v>
+        <v>255.913621478517</v>
       </c>
       <c r="H10" t="n">
-        <v>453.5492980307675</v>
+        <v>100.8931057727081</v>
       </c>
       <c r="I10" t="n">
-        <v>224.241542422005</v>
+        <v>209.1788911638618</v>
       </c>
       <c r="J10" t="n">
-        <v>224.0119019676069</v>
+        <v>285.8723420455359</v>
       </c>
       <c r="K10" t="n">
-        <v>328.0292642692195</v>
+        <v>326.09318403669</v>
       </c>
       <c r="L10" t="n">
-        <v>317.79303542216</v>
+        <v>419.7118462622228</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>8.882522817996928e-16</v>
+        <v>1.34276375726807e-16</v>
       </c>
       <c r="B11" t="n">
-        <v>-43.51395682176951</v>
+        <v>13.07169040182325</v>
       </c>
       <c r="C11" t="n">
-        <v>-29.97595638852331</v>
+        <v>0.268269752459522</v>
       </c>
       <c r="D11" t="n">
-        <v>-4.61627346876385</v>
+        <v>-0.2029426073998401</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.3844803120888034</v>
+        <v>-0.007829962003179071</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>431.454502347732</v>
+        <v>208.6496598163382</v>
       </c>
       <c r="H11" t="n">
-        <v>292.391012321192</v>
+        <v>202.1031213230056</v>
       </c>
       <c r="I11" t="n">
-        <v>268.4439002683727</v>
+        <v>336.6542068903365</v>
       </c>
       <c r="J11" t="n">
-        <v>425.3246468850106</v>
+        <v>130.8770012158401</v>
       </c>
       <c r="K11" t="n">
-        <v>367.9640033327566</v>
+        <v>326.1222458366921</v>
       </c>
       <c r="L11" t="n">
-        <v>198.9453684981033</v>
+        <v>352.7968951663149</v>
       </c>
     </row>
     <row r="12">
@@ -878,22 +878,22 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>300.1896575890655</v>
+        <v>159.8503687078877</v>
       </c>
       <c r="H12" t="n">
-        <v>460.4727091357807</v>
+        <v>187.48301332285</v>
       </c>
       <c r="I12" t="n">
-        <v>451.4362730085228</v>
+        <v>275.264103761584</v>
       </c>
       <c r="J12" t="n">
-        <v>175.3441372842708</v>
+        <v>236.1521574881101</v>
       </c>
       <c r="K12" t="n">
-        <v>247.3971304394904</v>
+        <v>447.90928881386</v>
       </c>
       <c r="L12" t="n">
-        <v>446.2664022331443</v>
+        <v>181.5026740474309</v>
       </c>
     </row>
     <row r="13">
@@ -916,22 +916,22 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>300.1896575890655</v>
+        <v>159.8503687078877</v>
       </c>
       <c r="H13" t="n">
-        <v>460.4727091357807</v>
+        <v>187.48301332285</v>
       </c>
       <c r="I13" t="n">
-        <v>451.4362730085228</v>
+        <v>275.264103761584</v>
       </c>
       <c r="J13" t="n">
-        <v>175.3441372842708</v>
+        <v>236.1521574881101</v>
       </c>
       <c r="K13" t="n">
-        <v>247.3971304394904</v>
+        <v>447.90928881386</v>
       </c>
       <c r="L13" t="n">
-        <v>446.2664022331443</v>
+        <v>181.5026740474309</v>
       </c>
     </row>
     <row r="14">
@@ -968,19 +968,19 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>9.940793884389218e-15</v>
+        <v>4.333519793092376e-16</v>
       </c>
       <c r="B15" t="n">
-        <v>66.02934538380599</v>
+        <v>18.22655570992734</v>
       </c>
       <c r="C15" t="n">
-        <v>31.23460795245</v>
+        <v>5.073828348551419</v>
       </c>
       <c r="D15" t="n">
-        <v>4.633267345186171</v>
+        <v>0.2031241998160949</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3845803842123143</v>
+        <v>0.007829107217133075</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
add motor module select output excel
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
@@ -480,458 +480,458 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4.333519793092376e-16</v>
+        <v>5.22721939457294e-15</v>
       </c>
       <c r="B2" t="n">
-        <v>14.32970207851291</v>
+        <v>30.06645133516072</v>
       </c>
       <c r="C2" t="n">
-        <v>3.866825595790485</v>
+        <v>15.41316595702082</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1867912526209001</v>
+        <v>5.499049262682917</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0008579083623691486</v>
+        <v>-0.03591399010017125</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>-0.8952622243621946</v>
       </c>
       <c r="G2" t="n">
-        <v>155.239055293018</v>
+        <v>161.8384480408196</v>
       </c>
       <c r="H2" t="n">
-        <v>268.7996574166283</v>
+        <v>125.220320322053</v>
       </c>
       <c r="I2" t="n">
-        <v>120.7042447589839</v>
+        <v>305.1915522490676</v>
       </c>
       <c r="J2" t="n">
-        <v>232.2635270345889</v>
+        <v>181.8882076851612</v>
       </c>
       <c r="K2" t="n">
-        <v>324.7167866562738</v>
+        <v>317.0375021962662</v>
       </c>
       <c r="L2" t="n">
-        <v>172.3554033854167</v>
+        <v>374.703450668515</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-4.626097186756907e-16</v>
+        <v>-6.204413142870467e-15</v>
       </c>
       <c r="B3" t="n">
-        <v>3.32380072754209</v>
+        <v>29.2197331618613</v>
       </c>
       <c r="C3" t="n">
-        <v>-3.612831347902668</v>
+        <v>15.23952006267491</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01203443264648458</v>
+        <v>3.880025475954377</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0005248379813055048</v>
+        <v>-0.4453597708064225</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>0.3298792650022951</v>
       </c>
       <c r="G3" t="n">
-        <v>126.298814844755</v>
+        <v>226.3340446830927</v>
       </c>
       <c r="H3" t="n">
-        <v>216.0676442175127</v>
+        <v>222.5272066889487</v>
       </c>
       <c r="I3" t="n">
-        <v>289.4538859265093</v>
+        <v>248.9685265380324</v>
       </c>
       <c r="J3" t="n">
-        <v>252.8933605583935</v>
+        <v>297.9954591804341</v>
       </c>
       <c r="K3" t="n">
-        <v>224.8385547745061</v>
+        <v>359.1705085651125</v>
       </c>
       <c r="L3" t="n">
-        <v>338.8836419862683</v>
+        <v>320.8349058227885</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5.831630857015175e-18</v>
+        <v>1.863956007164518e-16</v>
       </c>
       <c r="B4" t="n">
-        <v>18.22655570992734</v>
+        <v>32.05417989061412</v>
       </c>
       <c r="C4" t="n">
-        <v>5.055743683585101</v>
+        <v>17.30581623876991</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1955330917041322</v>
+        <v>5.66298790405206</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.007530158502224977</v>
+        <v>0.3178325223310227</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1.027399130741283</v>
       </c>
       <c r="G4" t="n">
-        <v>219.2313331751081</v>
+        <v>152.5727020577027</v>
       </c>
       <c r="H4" t="n">
-        <v>128.9995092647846</v>
+        <v>179.6064074381231</v>
       </c>
       <c r="I4" t="n">
-        <v>354.1295950808803</v>
+        <v>184.5045088657856</v>
       </c>
       <c r="J4" t="n">
-        <v>328.1288015049099</v>
+        <v>202.8836748547632</v>
       </c>
       <c r="K4" t="n">
-        <v>299.5968285520432</v>
+        <v>382.5681632395902</v>
       </c>
       <c r="L4" t="n">
-        <v>398.84889378004</v>
+        <v>431.38616872405</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1.660676677639394e-17</v>
+        <v>-3.223952492679939e-16</v>
       </c>
       <c r="B5" t="n">
-        <v>-9.122017648126123</v>
+        <v>-18.7786118921718</v>
       </c>
       <c r="C5" t="n">
-        <v>-5.057369306583921</v>
+        <v>-17.25829449094056</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1961165214039462</v>
+        <v>-5.610528988961049</v>
       </c>
       <c r="E5" t="n">
-        <v>0.00712352314118656</v>
+        <v>-0.1056833698240374</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>0.07239583186859895</v>
       </c>
       <c r="G5" t="n">
-        <v>94.73192944856265</v>
+        <v>124.3797192343261</v>
       </c>
       <c r="H5" t="n">
-        <v>164.9460680543654</v>
+        <v>256.3463377120632</v>
       </c>
       <c r="I5" t="n">
-        <v>276.7068012752046</v>
+        <v>140.6951223478019</v>
       </c>
       <c r="J5" t="n">
-        <v>209.4676251409578</v>
+        <v>212.7827444496326</v>
       </c>
       <c r="K5" t="n">
-        <v>251.6464575009193</v>
+        <v>443.4863764774395</v>
       </c>
       <c r="L5" t="n">
-        <v>187.6528711351712</v>
+        <v>189.3947636895273</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-6.465077602175565e-17</v>
+        <v>3.927569625436954e-15</v>
       </c>
       <c r="B6" t="n">
-        <v>12.54266116535535</v>
+        <v>31.50570731830327</v>
       </c>
       <c r="C6" t="n">
-        <v>5.073828348551419</v>
+        <v>17.35261166109319</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2028242187617373</v>
+        <v>5.717188834642265</v>
       </c>
       <c r="E6" t="n">
-        <v>0.003783973571307417</v>
+        <v>0.1736320610571605</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>0.7681607542222185</v>
       </c>
       <c r="G6" t="n">
-        <v>203.0457747057284</v>
+        <v>266.1201092733139</v>
       </c>
       <c r="H6" t="n">
-        <v>102.6348062425755</v>
+        <v>177.8712816698976</v>
       </c>
       <c r="I6" t="n">
-        <v>134.1890534089342</v>
+        <v>318.3118059139827</v>
       </c>
       <c r="J6" t="n">
-        <v>323.3941416316508</v>
+        <v>206.9325164888696</v>
       </c>
       <c r="K6" t="n">
-        <v>194.0390985245222</v>
+        <v>429.4411652083476</v>
       </c>
       <c r="L6" t="n">
-        <v>459.24388744721</v>
+        <v>164.162599667304</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9.780957829962677e-17</v>
+        <v>3.603874487490234e-16</v>
       </c>
       <c r="B7" t="n">
-        <v>-8.714835450147174</v>
+        <v>-8.619480675057829</v>
       </c>
       <c r="C7" t="n">
-        <v>-5.073926494032001</v>
+        <v>-17.34744887786591</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.202932551570449</v>
+        <v>-5.714493936043996</v>
       </c>
       <c r="E7" t="n">
-        <v>0.005647533378655745</v>
+        <v>-0.09907266370022728</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>0.03419362818375037</v>
       </c>
       <c r="G7" t="n">
-        <v>209.1811638258204</v>
+        <v>235.1385410379251</v>
       </c>
       <c r="H7" t="n">
-        <v>264.6011480012432</v>
+        <v>117.7234282677895</v>
       </c>
       <c r="I7" t="n">
-        <v>143.6996660999505</v>
+        <v>354.1582222563849</v>
       </c>
       <c r="J7" t="n">
-        <v>269.6116397426714</v>
+        <v>267.1660615540334</v>
       </c>
       <c r="K7" t="n">
-        <v>336.58436347155</v>
+        <v>287.4459374985538</v>
       </c>
       <c r="L7" t="n">
-        <v>206.0342853507156</v>
+        <v>414.1224681168188</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-1.092429492735409e-16</v>
+        <v>-4.265235481223306e-16</v>
       </c>
       <c r="B8" t="n">
-        <v>13.85418898014175</v>
+        <v>30.20354364453306</v>
       </c>
       <c r="C8" t="n">
-        <v>1.16787605292904</v>
+        <v>15.66575085829385</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2031241998160949</v>
+        <v>5.725802194098393</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0006447783890831559</v>
+        <v>-0.05466210476450293</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>-0.281370729313177</v>
       </c>
       <c r="G8" t="n">
-        <v>114.651205812829</v>
+        <v>214.2290962063973</v>
       </c>
       <c r="H8" t="n">
-        <v>252.8297301668283</v>
+        <v>210.4292745325691</v>
       </c>
       <c r="I8" t="n">
-        <v>323.0668816220197</v>
+        <v>154.5162790498206</v>
       </c>
       <c r="J8" t="n">
-        <v>357.506875532349</v>
+        <v>122.8354935177448</v>
       </c>
       <c r="K8" t="n">
-        <v>327.965826704513</v>
+        <v>210.1991076848735</v>
       </c>
       <c r="L8" t="n">
-        <v>194.9570618870869</v>
+        <v>469.7229076893103</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>3.633665321794214e-17</v>
+        <v>1.954424059435197e-17</v>
       </c>
       <c r="B9" t="n">
-        <v>11.01893040258089</v>
+        <v>-1.493950123935396</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.671335538621919</v>
+        <v>-16.24211173961427</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.2031258266151972</v>
+        <v>-5.726854380130433</v>
       </c>
       <c r="E9" t="n">
-        <v>1.785955698459928e-05</v>
+        <v>0.02955003778623009</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>0.02051080834873126</v>
       </c>
       <c r="G9" t="n">
-        <v>110.8629981366128</v>
+        <v>175.6593800771513</v>
       </c>
       <c r="H9" t="n">
-        <v>245.1752277991199</v>
+        <v>172.0168565498477</v>
       </c>
       <c r="I9" t="n">
-        <v>328.1722045891901</v>
+        <v>133.736916633457</v>
       </c>
       <c r="J9" t="n">
-        <v>284.4744390318555</v>
+        <v>243.2419600012682</v>
       </c>
       <c r="K9" t="n">
-        <v>193.9427140627287</v>
+        <v>241.1794543497848</v>
       </c>
       <c r="L9" t="n">
-        <v>200.6697782694127</v>
+        <v>235.8164765237252</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-5.533198564341929e-17</v>
+        <v>4.716377109975007e-16</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.9036399014302505</v>
+        <v>-6.802626014172191</v>
       </c>
       <c r="C10" t="n">
-        <v>-2.837660219235009</v>
+        <v>-15.59789541128376</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.202955857918495</v>
+        <v>-4.662538873505761</v>
       </c>
       <c r="E10" t="n">
-        <v>0.007829107217133075</v>
+        <v>1.157456477631696</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>0.01055761013205708</v>
       </c>
       <c r="G10" t="n">
-        <v>255.913621478517</v>
+        <v>127.370609012779</v>
       </c>
       <c r="H10" t="n">
-        <v>100.8931057727081</v>
+        <v>149.8294035551225</v>
       </c>
       <c r="I10" t="n">
-        <v>209.1788911638618</v>
+        <v>340.433793531568</v>
       </c>
       <c r="J10" t="n">
-        <v>285.8723420455359</v>
+        <v>347.8127476809043</v>
       </c>
       <c r="K10" t="n">
-        <v>326.09318403669</v>
+        <v>241.1023444973202</v>
       </c>
       <c r="L10" t="n">
-        <v>419.7118462622228</v>
+        <v>182.0130276525776</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1.34276375726807e-16</v>
+        <v>1.207217266449696e-16</v>
       </c>
       <c r="B11" t="n">
-        <v>13.07169040182325</v>
+        <v>-1.654728177146368</v>
       </c>
       <c r="C11" t="n">
-        <v>0.268269752459522</v>
+        <v>-3.284385825672477</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.2029426073998401</v>
+        <v>4.615263030867897</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.007829962003179071</v>
+        <v>-1.161557722577218</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>-0.04622155033688857</v>
       </c>
       <c r="G11" t="n">
-        <v>208.6496598163382</v>
+        <v>260.0808046287351</v>
       </c>
       <c r="H11" t="n">
-        <v>202.1031213230056</v>
+        <v>156.5454095064879</v>
       </c>
       <c r="I11" t="n">
-        <v>336.6542068903365</v>
+        <v>149.7946757665298</v>
       </c>
       <c r="J11" t="n">
-        <v>130.8770012158401</v>
+        <v>159.597325853146</v>
       </c>
       <c r="K11" t="n">
-        <v>326.1222458366921</v>
+        <v>479.6722043662787</v>
       </c>
       <c r="L11" t="n">
-        <v>352.7968951663149</v>
+        <v>336.6261433229088</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0</v>
+        <v>6.528211799254328e-16</v>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>3.408851763964884</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>-9.005323204467899</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>2.631560079710766</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>-0.318796193867298</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>1.096694142712799</v>
       </c>
       <c r="G12" t="n">
-        <v>159.8503687078877</v>
+        <v>220.8706434958923</v>
       </c>
       <c r="H12" t="n">
-        <v>187.48301332285</v>
+        <v>236.73461293662</v>
       </c>
       <c r="I12" t="n">
-        <v>275.264103761584</v>
+        <v>353.819113003415</v>
       </c>
       <c r="J12" t="n">
-        <v>236.1521574881101</v>
+        <v>179.303329809043</v>
       </c>
       <c r="K12" t="n">
-        <v>447.90928881386</v>
+        <v>235.6382834868263</v>
       </c>
       <c r="L12" t="n">
-        <v>181.5026740474309</v>
+        <v>466.5163839230927</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>-5.138086314245116e-16</v>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>24.24524056951606</v>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>9.698230191316881</v>
       </c>
       <c r="D13" t="n">
-        <v>0</v>
+        <v>-1.942114966058404</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>0.2558737290546119</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>-1.096783998556189</v>
       </c>
       <c r="G13" t="n">
-        <v>159.8503687078877</v>
+        <v>179.3382823031419</v>
       </c>
       <c r="H13" t="n">
-        <v>187.48301332285</v>
+        <v>257.7483544694285</v>
       </c>
       <c r="I13" t="n">
-        <v>275.264103761584</v>
+        <v>287.4560432481327</v>
       </c>
       <c r="J13" t="n">
-        <v>236.1521574881101</v>
+        <v>347.5738154698854</v>
       </c>
       <c r="K13" t="n">
-        <v>447.90928881386</v>
+        <v>308.4261324928663</v>
       </c>
       <c r="L13" t="n">
-        <v>181.5026740474309</v>
+        <v>183.5374916800037</v>
       </c>
     </row>
     <row r="14">
@@ -968,22 +968,22 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4.333519793092376e-16</v>
+        <v>5.22721939457294e-15</v>
       </c>
       <c r="B15" t="n">
-        <v>18.22655570992734</v>
+        <v>32.05417989061412</v>
       </c>
       <c r="C15" t="n">
-        <v>5.073828348551419</v>
+        <v>17.35261166109319</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2031241998160949</v>
+        <v>5.725802194098393</v>
       </c>
       <c r="E15" t="n">
-        <v>0.007829107217133075</v>
+        <v>1.157456477631696</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1.096694142712799</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add plot workspace test v1
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
@@ -480,382 +480,382 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>3.896714452764359e-16</v>
+        <v>4.369232328535308e-16</v>
       </c>
       <c r="B2" t="n">
-        <v>2.737554051798655</v>
+        <v>3.509234304586537</v>
       </c>
       <c r="C2" t="n">
-        <v>0.06986409927382436</v>
+        <v>0.02231472310047833</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1602253121937256</v>
+        <v>0.1984988493830444</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.002757997913445265</v>
+        <v>-0.005847353973372365</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>139.1624692475139</v>
+        <v>262.9309215257846</v>
       </c>
       <c r="H2" t="n">
-        <v>106.101773727676</v>
+        <v>250.593119041376</v>
       </c>
       <c r="I2" t="n">
-        <v>277.4607960838766</v>
+        <v>189.3466472338478</v>
       </c>
       <c r="J2" t="n">
-        <v>183.5356138239177</v>
+        <v>170.5234795881971</v>
       </c>
       <c r="K2" t="n">
-        <v>300.2555102547457</v>
+        <v>435.2884958741394</v>
       </c>
       <c r="L2" t="n">
-        <v>418.9762708994894</v>
+        <v>323.3535709215215</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-3.295355185473915e-16</v>
+        <v>-3.443652091672978e-16</v>
       </c>
       <c r="B3" t="n">
-        <v>5.497067341572366</v>
+        <v>4.348314216995742</v>
       </c>
       <c r="C3" t="n">
-        <v>0.932378557680911</v>
+        <v>0.7781640155346254</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.07674321454966482</v>
+        <v>0.05325486836358036</v>
       </c>
       <c r="E3" t="n">
-        <v>0.002251653634490288</v>
+        <v>-0.00208930724173994</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>222.8439743021924</v>
+        <v>161.0139463959628</v>
       </c>
       <c r="H3" t="n">
-        <v>226.1076609327292</v>
+        <v>114.3257286655506</v>
       </c>
       <c r="I3" t="n">
-        <v>159.6676690574295</v>
+        <v>237.6764467918796</v>
       </c>
       <c r="J3" t="n">
-        <v>359.6462063428085</v>
+        <v>157.9701713751696</v>
       </c>
       <c r="K3" t="n">
-        <v>241.6602823736781</v>
+        <v>338.1126726778903</v>
       </c>
       <c r="L3" t="n">
-        <v>261.1978359276691</v>
+        <v>171.6279553071195</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9.020282803053189e-19</v>
+        <v>-1.096151676971938e-16</v>
       </c>
       <c r="B4" t="n">
-        <v>7.267258419981797</v>
+        <v>7.275507434887453</v>
       </c>
       <c r="C4" t="n">
-        <v>2.158576295222186</v>
+        <v>2.15875806407584</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1957796907205593</v>
+        <v>0.1948114251957908</v>
       </c>
       <c r="E4" t="n">
-        <v>0.007255518498455599</v>
+        <v>0.006270868856277663</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>95.14499516009055</v>
+        <v>139.8692027260821</v>
       </c>
       <c r="H4" t="n">
-        <v>233.9689608005009</v>
+        <v>198.4484203120851</v>
       </c>
       <c r="I4" t="n">
-        <v>331.8563576416215</v>
+        <v>252.7341466287384</v>
       </c>
       <c r="J4" t="n">
-        <v>182.7442176710605</v>
+        <v>250.5544342742573</v>
       </c>
       <c r="K4" t="n">
-        <v>312.7598149390951</v>
+        <v>164.2193349486311</v>
       </c>
       <c r="L4" t="n">
-        <v>289.7143745797266</v>
+        <v>377.3897286667829</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-6.117474266014258e-17</v>
+        <v>-6.690592849368672e-17</v>
       </c>
       <c r="B5" t="n">
-        <v>-3.633766504446859</v>
+        <v>-3.660079684364874</v>
       </c>
       <c r="C5" t="n">
-        <v>-2.131500906967353</v>
+        <v>-2.119240722136432</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1688118667512442</v>
+        <v>-0.1968574971237458</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002156390022992584</v>
+        <v>0.004080059420644054</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>217.6336834131148</v>
+        <v>191.303160841143</v>
       </c>
       <c r="H5" t="n">
-        <v>224.5306576761033</v>
+        <v>180.5865156123098</v>
       </c>
       <c r="I5" t="n">
-        <v>261.6447977818998</v>
+        <v>267.3196705950712</v>
       </c>
       <c r="J5" t="n">
-        <v>292.1049828638553</v>
+        <v>147.629463253428</v>
       </c>
       <c r="K5" t="n">
-        <v>241.779662896094</v>
+        <v>438.9592208262376</v>
       </c>
       <c r="L5" t="n">
-        <v>355.1180756334485</v>
+        <v>345.842845662039</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>-1.055930742908061e-17</v>
+        <v>-6.541125813622848e-17</v>
       </c>
       <c r="B6" t="n">
-        <v>6.173514705675393</v>
+        <v>6.184280267216384</v>
       </c>
       <c r="C6" t="n">
-        <v>2.172317485627652</v>
+        <v>2.172360304770735</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2027027241466817</v>
+        <v>0.202888306899548</v>
       </c>
       <c r="E6" t="n">
-        <v>0.006636470843877285</v>
+        <v>0.006842554569799453</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>153.6074935304167</v>
+        <v>151.0384155741571</v>
       </c>
       <c r="H6" t="n">
-        <v>226.9016543952538</v>
+        <v>232.7419621731932</v>
       </c>
       <c r="I6" t="n">
-        <v>336.470339540183</v>
+        <v>257.6114779613218</v>
       </c>
       <c r="J6" t="n">
-        <v>258.0140376927241</v>
+        <v>169.5852684107635</v>
       </c>
       <c r="K6" t="n">
-        <v>470.5521282863169</v>
+        <v>268.1783266636024</v>
       </c>
       <c r="L6" t="n">
-        <v>405.6950453514312</v>
+        <v>262.4387458311487</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1.255896232806766e-17</v>
+        <v>1.119443035298385e-16</v>
       </c>
       <c r="B7" t="n">
-        <v>0.2051034198074366</v>
+        <v>0.9216233176434487</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.172544866685358</v>
+        <v>-2.172328915215547</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.2029742037666173</v>
+        <v>-0.202824541857372</v>
       </c>
       <c r="E7" t="n">
-        <v>0.007344350569165229</v>
+        <v>-0.003518574508551281</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>91.32774854755333</v>
+        <v>210.3202613961717</v>
       </c>
       <c r="H7" t="n">
-        <v>167.0767432473507</v>
+        <v>160.5938251362804</v>
       </c>
       <c r="I7" t="n">
-        <v>326.7948502760407</v>
+        <v>322.8635502028208</v>
       </c>
       <c r="J7" t="n">
-        <v>334.3775397079096</v>
+        <v>254.192471832567</v>
       </c>
       <c r="K7" t="n">
-        <v>425.8000464268531</v>
+        <v>221.3177177024994</v>
       </c>
       <c r="L7" t="n">
-        <v>354.9993669547285</v>
+        <v>285.4775941173374</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>-1.085217845472576e-16</v>
+        <v>1.141851182777251e-16</v>
       </c>
       <c r="B8" t="n">
-        <v>4.800307518608793</v>
+        <v>3.677916292224647</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.1355644008929682</v>
+        <v>-0.1405338142185297</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2031218468440417</v>
+        <v>0.2031216667433313</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0003151999537749535</v>
+        <v>0.0007774498665639034</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>130.4123435782047</v>
+        <v>90.79656676981155</v>
       </c>
       <c r="H8" t="n">
-        <v>221.7717244399619</v>
+        <v>234.1307011604318</v>
       </c>
       <c r="I8" t="n">
-        <v>213.1724318371147</v>
+        <v>191.9633015571191</v>
       </c>
       <c r="J8" t="n">
-        <v>234.7475776197601</v>
+        <v>278.0272657358925</v>
       </c>
       <c r="K8" t="n">
-        <v>169.2539968887581</v>
+        <v>208.6030515822439</v>
       </c>
       <c r="L8" t="n">
-        <v>210.4631843872227</v>
+        <v>296.5229552581735</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-3.072499163359244e-18</v>
+        <v>3.782068713035025e-17</v>
       </c>
       <c r="B9" t="n">
-        <v>-0.9567436167784098</v>
+        <v>5.150488181673553</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.945344244893715</v>
+        <v>0.04408566339922632</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.2031216631868815</v>
+        <v>-0.2031246564133402</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0007951444826114006</v>
+        <v>0.0007486420864025826</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>113.7575893067084</v>
+        <v>133.6862570489017</v>
       </c>
       <c r="H9" t="n">
-        <v>244.987381535725</v>
+        <v>158.3116013939234</v>
       </c>
       <c r="I9" t="n">
-        <v>341.588748707119</v>
+        <v>164.5697315079758</v>
       </c>
       <c r="J9" t="n">
-        <v>289.3378789733964</v>
+        <v>149.9922340813116</v>
       </c>
       <c r="K9" t="n">
-        <v>201.5798243302697</v>
+        <v>276.445576150904</v>
       </c>
       <c r="L9" t="n">
-        <v>202.5173681864425</v>
+        <v>270.1608059793848</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.518219360788948e-17</v>
+        <v>-7.520838023623159e-18</v>
       </c>
       <c r="B10" t="n">
-        <v>2.967641730304288</v>
+        <v>3.616759721407124</v>
       </c>
       <c r="C10" t="n">
-        <v>-2.097286627394027</v>
+        <v>-1.220394042897019</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.2029266557956295</v>
+        <v>-0.2029379341052776</v>
       </c>
       <c r="E10" t="n">
-        <v>0.007828880082645486</v>
+        <v>0.0078302274230879</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>132.8769030567743</v>
+        <v>262.1238657839883</v>
       </c>
       <c r="H10" t="n">
-        <v>258.6872592810095</v>
+        <v>260.7838098832204</v>
       </c>
       <c r="I10" t="n">
-        <v>139.1130445947136</v>
+        <v>265.3483843434504</v>
       </c>
       <c r="J10" t="n">
-        <v>292.157659285013</v>
+        <v>309.1625476027825</v>
       </c>
       <c r="K10" t="n">
-        <v>448.0945606398641</v>
+        <v>356.5473552379969</v>
       </c>
       <c r="L10" t="n">
-        <v>274.0920069477049</v>
+        <v>183.6233003785019</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1.568269645545887e-17</v>
+        <v>1.481746108223539e-16</v>
       </c>
       <c r="B11" t="n">
-        <v>5.695513254692193</v>
+        <v>4.23300683046463</v>
       </c>
       <c r="C11" t="n">
-        <v>1.434949470147667</v>
+        <v>-0.8185232967918817</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2029583521528772</v>
+        <v>0.2029508253962183</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.007830636951523761</v>
+        <v>-0.00783071971882288</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>209.616503710768</v>
+        <v>229.9114995385827</v>
       </c>
       <c r="H11" t="n">
-        <v>126.9719853100555</v>
+        <v>102.4426541791653</v>
       </c>
       <c r="I11" t="n">
-        <v>263.0752389717435</v>
+        <v>242.2950504597384</v>
       </c>
       <c r="J11" t="n">
-        <v>211.0447222529531</v>
+        <v>357.8141211899173</v>
       </c>
       <c r="K11" t="n">
-        <v>430.4404075677971</v>
+        <v>371.2053684897553</v>
       </c>
       <c r="L11" t="n">
-        <v>452.8460427179565</v>
+        <v>166.6124319102381</v>
       </c>
     </row>
     <row r="12">
@@ -878,22 +878,22 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>157.361466727191</v>
+        <v>92.37909454555187</v>
       </c>
       <c r="H12" t="n">
-        <v>187.3581448081296</v>
+        <v>233.2307720590494</v>
       </c>
       <c r="I12" t="n">
-        <v>294.438387671837</v>
+        <v>121.8987392643202</v>
       </c>
       <c r="J12" t="n">
-        <v>219.0052955025046</v>
+        <v>244.8174478316882</v>
       </c>
       <c r="K12" t="n">
-        <v>421.6591003189133</v>
+        <v>222.3005622628649</v>
       </c>
       <c r="L12" t="n">
-        <v>223.6863834221978</v>
+        <v>319.2995454049861</v>
       </c>
     </row>
     <row r="13">
@@ -916,22 +916,22 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>157.361466727191</v>
+        <v>92.37909454555187</v>
       </c>
       <c r="H13" t="n">
-        <v>187.3581448081296</v>
+        <v>233.2307720590494</v>
       </c>
       <c r="I13" t="n">
-        <v>294.438387671837</v>
+        <v>121.8987392643202</v>
       </c>
       <c r="J13" t="n">
-        <v>219.0052955025046</v>
+        <v>244.8174478316882</v>
       </c>
       <c r="K13" t="n">
-        <v>421.6591003189133</v>
+        <v>222.3005622628649</v>
       </c>
       <c r="L13" t="n">
-        <v>223.6863834221978</v>
+        <v>319.2995454049861</v>
       </c>
     </row>
     <row r="14">
@@ -968,19 +968,19 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3.896714452764359e-16</v>
+        <v>4.369232328535308e-16</v>
       </c>
       <c r="B15" t="n">
-        <v>7.267258419981797</v>
+        <v>7.275507434887453</v>
       </c>
       <c r="C15" t="n">
-        <v>2.172317485627652</v>
+        <v>2.172360304770735</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2031218468440417</v>
+        <v>0.2031216667433313</v>
       </c>
       <c r="E15" t="n">
-        <v>0.007828880082645486</v>
+        <v>0.0078302274230879</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
GUI set the joint angle limit ok
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
@@ -480,382 +480,382 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4.691782867654174e-16</v>
+        <v>4.063524445482365e-16</v>
       </c>
       <c r="B2" t="n">
-        <v>8.568828798017265</v>
+        <v>3.916541341086006</v>
       </c>
       <c r="C2" t="n">
-        <v>1.616416139369957</v>
+        <v>1.906077320652793</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1421025188292863</v>
+        <v>0.2028584521640072</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.004328396022916045</v>
+        <v>0.004925361909771284</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>215.0726248022922</v>
+        <v>-208.1745872777258</v>
       </c>
       <c r="H2" t="n">
-        <v>207.9346329650483</v>
+        <v>-203.0419183346576</v>
       </c>
       <c r="I2" t="n">
-        <v>169.9171209843221</v>
+        <v>-246.1550574309999</v>
       </c>
       <c r="J2" t="n">
-        <v>213.2018219615335</v>
+        <v>-146.6725370012521</v>
       </c>
       <c r="K2" t="n">
-        <v>193.7513158153378</v>
+        <v>-141.1177935318975</v>
       </c>
       <c r="L2" t="n">
-        <v>185.0806846688032</v>
+        <v>-279.9129905442529</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-4.450914406332993e-16</v>
+        <v>-3.368415777166166e-16</v>
       </c>
       <c r="B3" t="n">
-        <v>12.22227194583463</v>
+        <v>4.471184443022047</v>
       </c>
       <c r="C3" t="n">
-        <v>0.9591828464969584</v>
+        <v>0.1453697554498275</v>
       </c>
       <c r="D3" t="n">
-        <v>0.194875136789229</v>
+        <v>0.04873379862579773</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.005861963408374389</v>
+        <v>0.001273478104138466</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>196.7744509358578</v>
+        <v>-293.2294369792257</v>
       </c>
       <c r="H3" t="n">
-        <v>239.9901963770123</v>
+        <v>-120.0686845491362</v>
       </c>
       <c r="I3" t="n">
-        <v>306.3384403869329</v>
+        <v>-184.6342420815687</v>
       </c>
       <c r="J3" t="n">
-        <v>333.6972478704073</v>
+        <v>-147.6193050711527</v>
       </c>
       <c r="K3" t="n">
-        <v>276.518533793306</v>
+        <v>-105.8567527211622</v>
       </c>
       <c r="L3" t="n">
-        <v>267.520237700501</v>
+        <v>-144.6282402760124</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1.122363523840749e-16</v>
+        <v>1.704925907841156e-16</v>
       </c>
       <c r="B4" t="n">
-        <v>14.52488130032127</v>
+        <v>6.637260372540447</v>
       </c>
       <c r="C4" t="n">
-        <v>3.247643124697207</v>
+        <v>1.638484214475896</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1876757544393909</v>
+        <v>0.2030538491808176</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.005213900617646638</v>
+        <v>0.003529031722155214</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>131.2786099384052</v>
+        <v>-231.4652342148976</v>
       </c>
       <c r="H4" t="n">
-        <v>250.0317385949927</v>
+        <v>-144.9260177355144</v>
       </c>
       <c r="I4" t="n">
-        <v>244.3897665999187</v>
+        <v>-109.371194272712</v>
       </c>
       <c r="J4" t="n">
-        <v>165.0389639245632</v>
+        <v>-209.6727899851831</v>
       </c>
       <c r="K4" t="n">
-        <v>419.0759890310393</v>
+        <v>-287.0280676770373</v>
       </c>
       <c r="L4" t="n">
-        <v>207.6443914820977</v>
+        <v>-115.5911673879991</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>4.721721347937581e-17</v>
+        <v>9.671613097345813e-17</v>
       </c>
       <c r="B5" t="n">
-        <v>-6.693887947543552</v>
+        <v>-4.766466998461144</v>
       </c>
       <c r="C5" t="n">
-        <v>-3.212805837060288</v>
+        <v>-1.006881167702509</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1971534819961066</v>
+        <v>-0.1189107041234773</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.007561199417942482</v>
+        <v>-0.001890699315824726</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>99.42227809818651</v>
+        <v>-231.3221909900807</v>
       </c>
       <c r="H5" t="n">
-        <v>195.9041078689584</v>
+        <v>-123.9776782299967</v>
       </c>
       <c r="I5" t="n">
-        <v>174.2928910695422</v>
+        <v>-295.4473707277004</v>
       </c>
       <c r="J5" t="n">
-        <v>174.6185384676436</v>
+        <v>-143.2152345712038</v>
       </c>
       <c r="K5" t="n">
-        <v>347.0606765947147</v>
+        <v>-179.8649574859882</v>
       </c>
       <c r="L5" t="n">
-        <v>293.9047343562585</v>
+        <v>-259.3292697400526</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1.108359113476444e-16</v>
+        <v>5.144069548575249e-17</v>
       </c>
       <c r="B6" t="n">
-        <v>8.609332028616155</v>
+        <v>-0.5197585358209855</v>
       </c>
       <c r="C6" t="n">
-        <v>3.271628708323247</v>
+        <v>2.17264233183042</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2029811892417671</v>
+        <v>0.2030268927719243</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.005470099100115373</v>
+        <v>0.004156656352952934</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>206.2356115480653</v>
+        <v>-272.4871604646153</v>
       </c>
       <c r="H6" t="n">
-        <v>163.1217528687789</v>
+        <v>-280.9303057016181</v>
       </c>
       <c r="I6" t="n">
-        <v>217.7026266429486</v>
+        <v>-276.4034253494459</v>
       </c>
       <c r="J6" t="n">
-        <v>333.9796511443623</v>
+        <v>-104.6192128118125</v>
       </c>
       <c r="K6" t="n">
-        <v>439.9903235221292</v>
+        <v>-179.6040244803747</v>
       </c>
       <c r="L6" t="n">
-        <v>364.8366764151382</v>
+        <v>-269.5248598955652</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>-7.619972966221606e-17</v>
+        <v>-4.303938579808872e-17</v>
       </c>
       <c r="B7" t="n">
-        <v>7.821222951528544</v>
+        <v>2.923377079033285</v>
       </c>
       <c r="C7" t="n">
-        <v>-3.272803933977945</v>
+        <v>-2.172596314265808</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.2030562642183016</v>
+        <v>-0.2030119275769316</v>
       </c>
       <c r="E7" t="n">
-        <v>0.003066269570319326</v>
+        <v>-0.005451478560159417</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>90.10220990597134</v>
+        <v>-151.1712455560321</v>
       </c>
       <c r="H7" t="n">
-        <v>175.4012366729903</v>
+        <v>-271.6705838337439</v>
       </c>
       <c r="I7" t="n">
-        <v>247.5442017662156</v>
+        <v>-256.7060963646106</v>
       </c>
       <c r="J7" t="n">
-        <v>247.3207607780483</v>
+        <v>-142.1653804239488</v>
       </c>
       <c r="K7" t="n">
-        <v>258.3020309745055</v>
+        <v>-279.0205017488011</v>
       </c>
       <c r="L7" t="n">
-        <v>319.1957959478577</v>
+        <v>-185.061471328837</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1.444710257344163e-16</v>
+        <v>7.833661742275462e-17</v>
       </c>
       <c r="B8" t="n">
-        <v>13.23818167121957</v>
+        <v>-1.440363643336592</v>
       </c>
       <c r="C8" t="n">
-        <v>3.168248782096023</v>
+        <v>2.152773694730953</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2031215892242177</v>
+        <v>0.2031247678598138</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0007705572033509834</v>
+        <v>-0.0002946371425437736</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>261.4556162229031</v>
+        <v>-183.8988453315329</v>
       </c>
       <c r="H8" t="n">
-        <v>129.501214935772</v>
+        <v>-280.9776195213938</v>
       </c>
       <c r="I8" t="n">
-        <v>197.0030793097069</v>
+        <v>-103.5165858071256</v>
       </c>
       <c r="J8" t="n">
-        <v>170.8877595913928</v>
+        <v>-194.5448059550203</v>
       </c>
       <c r="K8" t="n">
-        <v>322.9484908073283</v>
+        <v>-224.658804549328</v>
       </c>
       <c r="L8" t="n">
-        <v>203.6389310009046</v>
+        <v>-118.760409201183</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-5.207520243766e-17</v>
+        <v>6.504622165983421e-17</v>
       </c>
       <c r="B9" t="n">
-        <v>7.308640482386348</v>
+        <v>2.875417210005948</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.890713208275677</v>
+        <v>-2.002641016924062</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.2031255278670108</v>
+        <v>-0.203123901232551</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.0002886131224947452</v>
+        <v>0.000937797406897592</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>151.3455260350566</v>
+        <v>-140.8275831216113</v>
       </c>
       <c r="H9" t="n">
-        <v>169.9392146678988</v>
+        <v>-246.2728678862812</v>
       </c>
       <c r="I9" t="n">
-        <v>242.5740183442258</v>
+        <v>-196.5882572474681</v>
       </c>
       <c r="J9" t="n">
-        <v>218.2885218675283</v>
+        <v>-189.3672629472696</v>
       </c>
       <c r="K9" t="n">
-        <v>392.5067068395122</v>
+        <v>-220.0206695226231</v>
       </c>
       <c r="L9" t="n">
-        <v>230.2287898764592</v>
+        <v>-133.861951162339</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-1.328197186547799e-17</v>
+        <v>-1.863651697540624e-16</v>
       </c>
       <c r="B10" t="n">
-        <v>5.222484323557057</v>
+        <v>0.5826893957639101</v>
       </c>
       <c r="C10" t="n">
-        <v>0.16341457459317</v>
+        <v>-1.673756150158109</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.2029586363114567</v>
+        <v>0.2029583035456022</v>
       </c>
       <c r="E10" t="n">
-        <v>0.007830578738937497</v>
+        <v>0.007829986794926467</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>138.5366066680242</v>
+        <v>-154.39409998759</v>
       </c>
       <c r="H10" t="n">
-        <v>184.9247285901325</v>
+        <v>-262.8754186897602</v>
       </c>
       <c r="I10" t="n">
-        <v>162.9318341934817</v>
+        <v>-182.7291684390804</v>
       </c>
       <c r="J10" t="n">
-        <v>331.0159851404583</v>
+        <v>-210.2113947718159</v>
       </c>
       <c r="K10" t="n">
-        <v>213.2772426807919</v>
+        <v>-269.209651321293</v>
       </c>
       <c r="L10" t="n">
-        <v>202.1940897674032</v>
+        <v>-298.6447000845739</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>3.312986342686658e-17</v>
+        <v>-3.306700140884343e-17</v>
       </c>
       <c r="B11" t="n">
-        <v>-6.626484897976594</v>
+        <v>0.366540782828827</v>
       </c>
       <c r="C11" t="n">
-        <v>-3.271638413694874</v>
+        <v>1.476312830276173</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.2029555104888276</v>
+        <v>-0.2028757409776071</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.007830837554917902</v>
+        <v>-0.007823538990350171</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>222.9971680034504</v>
+        <v>-281.3685620372889</v>
       </c>
       <c r="H11" t="n">
-        <v>99.66364827678171</v>
+        <v>-280.4087536240257</v>
       </c>
       <c r="I11" t="n">
-        <v>275.51551458747</v>
+        <v>-282.6744295386466</v>
       </c>
       <c r="J11" t="n">
-        <v>144.309693780466</v>
+        <v>-220.6441498996765</v>
       </c>
       <c r="K11" t="n">
-        <v>186.9632134486625</v>
+        <v>-236.6576908197543</v>
       </c>
       <c r="L11" t="n">
-        <v>414.3098471159769</v>
+        <v>-206.0416915890776</v>
       </c>
     </row>
     <row r="12">
@@ -878,22 +878,22 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>204.4582406589592</v>
+        <v>-172.7103297485407</v>
       </c>
       <c r="H12" t="n">
-        <v>230.5089505503077</v>
+        <v>-186.3159208167994</v>
       </c>
       <c r="I12" t="n">
-        <v>246.8543434508836</v>
+        <v>-110.1601648855138</v>
       </c>
       <c r="J12" t="n">
-        <v>252.5665560363857</v>
+        <v>-275.0342298516327</v>
       </c>
       <c r="K12" t="n">
-        <v>275.8901355628469</v>
+        <v>-189.4738739884041</v>
       </c>
       <c r="L12" t="n">
-        <v>214.1734481962645</v>
+        <v>-249.3092308006451</v>
       </c>
     </row>
     <row r="13">
@@ -916,22 +916,22 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>204.4582406589592</v>
+        <v>-172.7103297485407</v>
       </c>
       <c r="H13" t="n">
-        <v>230.5089505503077</v>
+        <v>-186.3159208167994</v>
       </c>
       <c r="I13" t="n">
-        <v>246.8543434508836</v>
+        <v>-110.1601648855138</v>
       </c>
       <c r="J13" t="n">
-        <v>252.5665560363857</v>
+        <v>-275.0342298516327</v>
       </c>
       <c r="K13" t="n">
-        <v>275.8901355628469</v>
+        <v>-189.4738739884041</v>
       </c>
       <c r="L13" t="n">
-        <v>214.1734481962645</v>
+        <v>-249.3092308006451</v>
       </c>
     </row>
     <row r="14">
@@ -968,19 +968,19 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4.691782867654174e-16</v>
+        <v>4.063524445482365e-16</v>
       </c>
       <c r="B15" t="n">
-        <v>14.52488130032127</v>
+        <v>6.637260372540447</v>
       </c>
       <c r="C15" t="n">
-        <v>3.271628708323247</v>
+        <v>2.17264233183042</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2031215892242177</v>
+        <v>0.2031247678598138</v>
       </c>
       <c r="E15" t="n">
-        <v>0.007830578738937497</v>
+        <v>0.007829986794926467</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
add traject torque pos vel acc output excel ok
</commit_message>
<xml_diff>
--- a/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
+++ b/dynamics/src/dynamics/xlsx/dynamics_static_torque_calc.xlsx
@@ -480,382 +480,382 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>4.73722504211298e-16</v>
+        <v>4.091402219407377e-16</v>
       </c>
       <c r="B2" t="n">
-        <v>3.203646115624323</v>
+        <v>3.055503303417273</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1112259055405668</v>
+        <v>1.732034947384396</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.1690734890510618</v>
+        <v>0.2007802082634225</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.003163778220487342</v>
+        <v>0.006188644216855313</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>-499.6639982249136</v>
+        <v>235.2212983451001</v>
       </c>
       <c r="H2" t="n">
-        <v>-297.5173022443434</v>
+        <v>154.1500158816395</v>
       </c>
       <c r="I2" t="n">
-        <v>-309.7916347825311</v>
+        <v>229.9827586967068</v>
       </c>
       <c r="J2" t="n">
-        <v>-190.7921793328458</v>
+        <v>243.3897731718233</v>
       </c>
       <c r="K2" t="n">
-        <v>-300.9147235258574</v>
+        <v>194.9519682072257</v>
       </c>
       <c r="L2" t="n">
-        <v>-192.4814796218298</v>
+        <v>212.2485290368783</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>-3.562064473787729e-16</v>
+        <v>-3.803898399444096e-16</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.3778973661195459</v>
+        <v>1.946855554106047</v>
       </c>
       <c r="C3" t="n">
-        <v>-1.841218599707578</v>
+        <v>-1.843759210184875</v>
       </c>
       <c r="D3" t="n">
-        <v>0.1274363478919197</v>
+        <v>-0.1835493982994691</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.004907047384638874</v>
+        <v>-0.001993192841362582</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>-350.7198558091643</v>
+        <v>283.2323755089495</v>
       </c>
       <c r="H3" t="n">
-        <v>-489.371102776032</v>
+        <v>224.5044515745452</v>
       </c>
       <c r="I3" t="n">
-        <v>-509.7329763362149</v>
+        <v>268.5686654715594</v>
       </c>
       <c r="J3" t="n">
-        <v>-493.7933328382941</v>
+        <v>229.2500578626596</v>
       </c>
       <c r="K3" t="n">
-        <v>-440.8948219099566</v>
+        <v>107.27284664215</v>
       </c>
       <c r="L3" t="n">
-        <v>-287.8203541825995</v>
+        <v>171.7695117972128</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5.072228343796878e-19</v>
+        <v>-1.087024124102577e-16</v>
       </c>
       <c r="B4" t="n">
-        <v>7.26081075774644</v>
+        <v>6.383847962420203</v>
       </c>
       <c r="C4" t="n">
-        <v>2.14569648205008</v>
+        <v>1.415453782885952</v>
       </c>
       <c r="D4" t="n">
-        <v>0.20294743746403</v>
+        <v>0.2023303041251349</v>
       </c>
       <c r="E4" t="n">
-        <v>0.007557603389631859</v>
+        <v>-0.001591208748088253</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>-506.0309371605395</v>
+        <v>252.6791327241024</v>
       </c>
       <c r="H4" t="n">
-        <v>-469.9469895841947</v>
+        <v>142.127360533965</v>
       </c>
       <c r="I4" t="n">
-        <v>-295.3194117376828</v>
+        <v>112.0213867593917</v>
       </c>
       <c r="J4" t="n">
-        <v>-205.787225671946</v>
+        <v>296.1932018227483</v>
       </c>
       <c r="K4" t="n">
-        <v>-381.7681230526977</v>
+        <v>150.9117578934941</v>
       </c>
       <c r="L4" t="n">
-        <v>-235.7430068630212</v>
+        <v>285.1692146299674</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>-5.73943524479858e-17</v>
+        <v>-2.471585942156827e-16</v>
       </c>
       <c r="B5" t="n">
-        <v>-7.283282190053392</v>
+        <v>-3.129840262806506</v>
       </c>
       <c r="C5" t="n">
-        <v>-2.167405347830383</v>
+        <v>-2.063680658162722</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.2027763146522337</v>
+        <v>-0.1930767728255319</v>
       </c>
       <c r="E5" t="n">
-        <v>0.002558937438751546</v>
+        <v>0.001206372564489008</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>-496.5530644694226</v>
+        <v>294.0521716091692</v>
       </c>
       <c r="H5" t="n">
-        <v>-408.9005457756559</v>
+        <v>105.8680120567771</v>
       </c>
       <c r="I5" t="n">
-        <v>-519.0327803835905</v>
+        <v>247.8094856972645</v>
       </c>
       <c r="J5" t="n">
-        <v>-385.2717196060852</v>
+        <v>206.449247629462</v>
       </c>
       <c r="K5" t="n">
-        <v>-323.9081466033732</v>
+        <v>134.8578781631891</v>
       </c>
       <c r="L5" t="n">
-        <v>-316.572133186045</v>
+        <v>128.707964038932</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6.492392646159016e-17</v>
+        <v>-3.225264426106674e-17</v>
       </c>
       <c r="B6" t="n">
-        <v>1.966854080322581</v>
+        <v>4.232745308826818</v>
       </c>
       <c r="C6" t="n">
-        <v>2.172577999215413</v>
+        <v>2.172130662493426</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2029629427194879</v>
+        <v>0.2026488309358206</v>
       </c>
       <c r="E6" t="n">
-        <v>0.00769698499555313</v>
+        <v>0.007817997588955489</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>-383.494104373841</v>
+        <v>263.4537320582812</v>
       </c>
       <c r="H6" t="n">
-        <v>-461.3585166405889</v>
+        <v>179.2151207829241</v>
       </c>
       <c r="I6" t="n">
-        <v>-219.9613106061616</v>
+        <v>287.7332103150164</v>
       </c>
       <c r="J6" t="n">
-        <v>-385.3282108315169</v>
+        <v>114.8845833110092</v>
       </c>
       <c r="K6" t="n">
-        <v>-335.4290792720597</v>
+        <v>178.2047393955353</v>
       </c>
       <c r="L6" t="n">
-        <v>-249.8164364632563</v>
+        <v>283.4299800911605</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8.517657641402115e-17</v>
+        <v>-1.198172884133362e-16</v>
       </c>
       <c r="B7" t="n">
-        <v>-6.768054021058761</v>
+        <v>2.576064671916451</v>
       </c>
       <c r="C7" t="n">
-        <v>-2.172451127473945</v>
+        <v>-2.172516786081878</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.2028351443973495</v>
+        <v>-0.2029358350451315</v>
       </c>
       <c r="E7" t="n">
-        <v>0.007609877777676778</v>
+        <v>-0.004911098508484864</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>-474.595004708436</v>
+        <v>121.7487930734277</v>
       </c>
       <c r="H7" t="n">
-        <v>-449.0695101145917</v>
+        <v>142.6316026076196</v>
       </c>
       <c r="I7" t="n">
-        <v>-268.191622531273</v>
+        <v>138.4936312060727</v>
       </c>
       <c r="J7" t="n">
-        <v>-278.153382999218</v>
+        <v>194.0098947973537</v>
       </c>
       <c r="K7" t="n">
-        <v>-383.5230840252482</v>
+        <v>133.1386858321638</v>
       </c>
       <c r="L7" t="n">
-        <v>-413.0153194489037</v>
+        <v>180.7483017453656</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2.004757525137446e-18</v>
+        <v>-2.672298253781471e-17</v>
       </c>
       <c r="B8" t="n">
-        <v>0.3727023865615509</v>
+        <v>4.549693012353724</v>
       </c>
       <c r="C8" t="n">
-        <v>-1.357975495517268</v>
+        <v>-0.563372943088447</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2031252960299102</v>
+        <v>0.2031052586107497</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.0005554946603836265</v>
+        <v>0.001946466232204936</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>-329.9706397558758</v>
+        <v>127.7573892925534</v>
       </c>
       <c r="H8" t="n">
-        <v>-498.9415031735107</v>
+        <v>283.5229704323186</v>
       </c>
       <c r="I8" t="n">
-        <v>-427.5409927701043</v>
+        <v>109.1967867457293</v>
       </c>
       <c r="J8" t="n">
-        <v>-348.14410930067</v>
+        <v>232.317487024862</v>
       </c>
       <c r="K8" t="n">
-        <v>-382.6306412535364</v>
+        <v>198.0156415859207</v>
       </c>
       <c r="L8" t="n">
-        <v>-450.3146390615858</v>
+        <v>299.4690796159133</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>-1.309099387540103e-17</v>
+        <v>-8.82585860985017e-17</v>
       </c>
       <c r="B9" t="n">
-        <v>-2.933489846937681</v>
+        <v>-1.441372094549233</v>
       </c>
       <c r="C9" t="n">
-        <v>1.69363384721638</v>
+        <v>-1.849935776345166</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.2031254140237084</v>
+        <v>-0.203113010028629</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0005501575069012728</v>
+        <v>-0.002203801592632328</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>-323.3509112766465</v>
+        <v>176.4130725822592</v>
       </c>
       <c r="H9" t="n">
-        <v>-203.9116710882615</v>
+        <v>245.713050886135</v>
       </c>
       <c r="I9" t="n">
-        <v>-188.5270732283834</v>
+        <v>117.1596281347101</v>
       </c>
       <c r="J9" t="n">
-        <v>-403.7532756405058</v>
+        <v>288.8138278404767</v>
       </c>
       <c r="K9" t="n">
-        <v>-342.519767073772</v>
+        <v>258.0456512981706</v>
       </c>
       <c r="L9" t="n">
-        <v>-354.5526215274361</v>
+        <v>248.8715905944032</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>-4.904102634856947e-17</v>
+        <v>1.403255602090964e-16</v>
       </c>
       <c r="B10" t="n">
-        <v>-4.427164329541238</v>
+        <v>3.594878788844059</v>
       </c>
       <c r="C10" t="n">
-        <v>0.5411657140883134</v>
+        <v>2.16522938234038</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.2029336637974995</v>
+        <v>0.2029505616889527</v>
       </c>
       <c r="E10" t="n">
-        <v>0.007830098411700369</v>
+        <v>0.007828303734870886</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>-364.2319640904965</v>
+        <v>168.0841434123181</v>
       </c>
       <c r="H10" t="n">
-        <v>-277.6036759814451</v>
+        <v>228.7006329939168</v>
       </c>
       <c r="I10" t="n">
-        <v>-393.920835950113</v>
+        <v>245.7353302695956</v>
       </c>
       <c r="J10" t="n">
-        <v>-205.7799248992835</v>
+        <v>125.1154989629193</v>
       </c>
       <c r="K10" t="n">
-        <v>-308.6816402879103</v>
+        <v>134.9351659490707</v>
       </c>
       <c r="L10" t="n">
-        <v>-520.9276900782138</v>
+        <v>264.6585282886405</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>-6.908124352411057e-17</v>
+        <v>-5.998515593512319e-17</v>
       </c>
       <c r="B11" t="n">
-        <v>-3.394597066631371</v>
+        <v>-2.79276373427344</v>
       </c>
       <c r="C11" t="n">
-        <v>1.671379403411398</v>
+        <v>-2.143502973102945</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.2029509325082046</v>
+        <v>-0.2029569121361087</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.0078277050484522</v>
+        <v>-0.007830464215228134</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>-200.2469639188261</v>
+        <v>103.1660510073546</v>
       </c>
       <c r="H11" t="n">
-        <v>-229.498715681002</v>
+        <v>283.2681422643896</v>
       </c>
       <c r="I11" t="n">
-        <v>-361.7276882958779</v>
+        <v>149.5838285754555</v>
       </c>
       <c r="J11" t="n">
-        <v>-401.1609552053811</v>
+        <v>280.7465981665982</v>
       </c>
       <c r="K11" t="n">
-        <v>-450.3089049203305</v>
+        <v>164.6393742083581</v>
       </c>
       <c r="L11" t="n">
-        <v>-297.3579742304087</v>
+        <v>267.6604337665934</v>
       </c>
     </row>
     <row r="12">
@@ -878,22 +878,22 @@
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>-289.2883895482012</v>
+        <v>217.577369532687</v>
       </c>
       <c r="H12" t="n">
-        <v>-177.8553582262861</v>
+        <v>179.3695940583734</v>
       </c>
       <c r="I12" t="n">
-        <v>-230.700804448371</v>
+        <v>282.4701161580262</v>
       </c>
       <c r="J12" t="n">
-        <v>-186.818658866641</v>
+        <v>242.819519033292</v>
       </c>
       <c r="K12" t="n">
-        <v>-208.9755097582397</v>
+        <v>169.0397098943142</v>
       </c>
       <c r="L12" t="n">
-        <v>-463.4017058426597</v>
+        <v>266.3169533656837</v>
       </c>
     </row>
     <row r="13">
@@ -916,22 +916,22 @@
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>-289.2883895482012</v>
+        <v>217.577369532687</v>
       </c>
       <c r="H13" t="n">
-        <v>-177.8553582262861</v>
+        <v>179.3695940583734</v>
       </c>
       <c r="I13" t="n">
-        <v>-230.700804448371</v>
+        <v>282.4701161580262</v>
       </c>
       <c r="J13" t="n">
-        <v>-186.818658866641</v>
+        <v>242.819519033292</v>
       </c>
       <c r="K13" t="n">
-        <v>-208.9755097582397</v>
+        <v>169.0397098943142</v>
       </c>
       <c r="L13" t="n">
-        <v>-463.4017058426597</v>
+        <v>266.3169533656837</v>
       </c>
     </row>
     <row r="14">
@@ -968,19 +968,19 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>4.73722504211298e-16</v>
+        <v>4.091402219407377e-16</v>
       </c>
       <c r="B15" t="n">
-        <v>7.26081075774644</v>
+        <v>6.383847962420203</v>
       </c>
       <c r="C15" t="n">
-        <v>2.172577999215413</v>
+        <v>2.172130662493426</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2031252960299102</v>
+        <v>0.2031052586107497</v>
       </c>
       <c r="E15" t="n">
-        <v>0.007830098411700369</v>
+        <v>0.007828303734870886</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>

</xml_diff>